<commit_message>
Mise à jour vers le nouveau template d'HL7 International (#50)
* test template2

* test template 2

* test template 2

* test template 2

* test template 2

* update index

* Add English language option to configuration

* Disable i18n-lang parameter in sushi-config.yaml

Comment out the i18n-lang parameter in the configuration.

* Update default language to 'fr-FR' in config

* Update sushi-config.yaml

* Enable English as an additional language option

* Rm english language

* add eng lang

* add translations & update scripts

* update

* update flga

* update sushi config

* update

* update sushi config

* add xp params

* update

* update

* Add translationinfo page (FR base + EN translation)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>

* update

* update

* update sushi-config

* update

* update ihe careteam

* Update ig.ini

* Update features.yml

---------

Co-authored-by: Claude Sonnet 4.6 <noreply@anthropic.com> ae492b350066b57aae9f83b6aabc577563e1a631
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-cds-bundle-response-recherche.xlsx
+++ b/main/ig/StructureDefinition-cds-bundle-response-recherche.xlsx
@@ -57,25 +57,25 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-12-03T08:47:15+00:00</t>
+    <t>2026-06-01T14:15:31+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
   </si>
   <si>
-    <t>ANS</t>
+    <t>Agence du Numérique en Santé (ANS) - 2-10 Rue d'Oradour-sur-Glane, 75015 Paris</t>
   </si>
   <si>
     <t>Contact</t>
   </si>
   <si>
-    <t>ANS (https://esante.gouv.fr)</t>
+    <t>Agence du Numérique en Santé (ANS) - 2-10 Rue d'Oradour-sur-Glane, 75015 Paris (https://esante.gouv.fr)</t>
   </si>
   <si>
     <t>Jurisdiction</t>
   </si>
   <si>
-    <t>FRANCE</t>
+    <t>France (la)</t>
   </si>
   <si>
     <t>Description</t>

</xml_diff>